<commit_message>
fix: add 's' to word success
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -423,9 +423,6 @@
     <t>concept</t>
   </si>
   <si>
-    <t>succes</t>
-  </si>
-  <si>
     <t>SingleStudentsNearby</t>
   </si>
   <si>
@@ -643,6 +640,9 @@
   </si>
   <si>
     <t>PrincessPhotoGuys</t>
+  </si>
+  <si>
+    <t>success</t>
   </si>
 </sst>
 </file>
@@ -1000,7 +1000,7 @@
         <v>21</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>134</v>
+        <v>207</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.2">
@@ -1008,7 +1008,7 @@
         <v>22</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C2" s="1">
         <v>820</v>
@@ -1083,7 +1083,7 @@
         <v>27</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C3" s="1">
         <v>820</v>
@@ -1155,7 +1155,7 @@
         <v>29</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C4" s="1">
         <v>820</v>
@@ -1224,7 +1224,7 @@
         <v>31</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C5" s="1">
         <v>820</v>
@@ -1296,7 +1296,7 @@
         <v>32</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C6" s="1">
         <v>820</v>
@@ -1365,7 +1365,7 @@
         <v>33</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C7" s="1">
         <v>820</v>
@@ -1434,7 +1434,7 @@
         <v>34</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C8" s="1">
         <v>820</v>
@@ -1503,7 +1503,7 @@
         <v>35</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C9" s="1">
         <v>820</v>
@@ -1572,7 +1572,7 @@
         <v>36</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C10" s="1">
         <v>820</v>
@@ -1641,7 +1641,7 @@
         <v>37</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C11" s="1">
         <v>820</v>
@@ -1710,7 +1710,7 @@
         <v>38</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C12" s="1">
         <v>820</v>
@@ -1779,7 +1779,7 @@
         <v>39</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C13" s="1">
         <v>820</v>
@@ -1854,7 +1854,7 @@
         <v>41</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C14" s="1">
         <v>820</v>
@@ -1926,7 +1926,7 @@
         <v>42</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C15" s="1">
         <v>820</v>
@@ -2001,7 +2001,7 @@
         <v>43</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C16" s="1">
         <v>820</v>
@@ -2073,7 +2073,7 @@
         <v>44</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C17" s="1">
         <v>820</v>
@@ -2145,7 +2145,7 @@
         <v>45</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C18" s="1">
         <v>820</v>
@@ -2217,7 +2217,7 @@
         <v>46</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C19" s="1">
         <v>820</v>
@@ -2289,7 +2289,7 @@
         <v>47</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C20" s="1">
         <v>820</v>
@@ -2361,7 +2361,7 @@
         <v>48</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C21" s="1">
         <v>820</v>
@@ -2433,7 +2433,7 @@
         <v>49</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C22" s="1">
         <v>820</v>
@@ -2505,7 +2505,7 @@
         <v>50</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C23" s="1">
         <v>820</v>
@@ -2577,7 +2577,7 @@
         <v>51</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C24" s="1">
         <v>820</v>
@@ -2649,7 +2649,7 @@
         <v>52</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C25" s="1">
         <v>820</v>
@@ -2721,7 +2721,7 @@
         <v>53</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C26" s="1">
         <v>820</v>
@@ -2793,7 +2793,7 @@
         <v>54</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C27" s="1">
         <v>869</v>
@@ -2868,7 +2868,7 @@
         <v>56</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C28" s="1">
         <v>869</v>
@@ -2943,7 +2943,7 @@
         <v>57</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C29" s="1">
         <v>869</v>
@@ -3018,7 +3018,7 @@
         <v>58</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C30" s="1">
         <v>869</v>
@@ -3093,7 +3093,7 @@
         <v>59</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C31" s="1">
         <v>869</v>
@@ -3165,7 +3165,7 @@
         <v>60</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C32" s="1">
         <v>869</v>
@@ -3237,7 +3237,7 @@
         <v>61</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C33" s="1">
         <v>869</v>
@@ -3312,7 +3312,7 @@
         <v>62</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C34" s="1">
         <v>869</v>
@@ -3384,7 +3384,7 @@
         <v>63</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C35" s="1">
         <v>869</v>
@@ -3456,7 +3456,7 @@
         <v>64</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C36" s="1">
         <v>869</v>
@@ -3528,7 +3528,7 @@
         <v>65</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C37" s="1">
         <v>869</v>
@@ -3600,7 +3600,7 @@
         <v>66</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C38" s="1">
         <v>869</v>
@@ -3672,7 +3672,7 @@
         <v>67</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C39" s="1">
         <v>869</v>
@@ -3747,7 +3747,7 @@
         <v>68</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C40" s="1">
         <v>869</v>
@@ -3819,7 +3819,7 @@
         <v>69</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C41" s="1">
         <v>869</v>
@@ -3894,7 +3894,7 @@
         <v>70</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C42" s="1">
         <v>869</v>
@@ -3966,7 +3966,7 @@
         <v>71</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C43" s="1">
         <v>869</v>
@@ -4038,7 +4038,7 @@
         <v>72</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C44" s="1">
         <v>869</v>
@@ -4113,7 +4113,7 @@
         <v>73</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C45" s="1">
         <v>869</v>
@@ -4185,7 +4185,7 @@
         <v>74</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C46" s="1">
         <v>743</v>
@@ -4260,7 +4260,7 @@
         <v>77</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C47" s="1">
         <v>743</v>
@@ -4335,7 +4335,7 @@
         <v>78</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C48" s="1">
         <v>743</v>
@@ -4410,7 +4410,7 @@
         <v>79</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C49" s="1">
         <v>743</v>
@@ -4485,7 +4485,7 @@
         <v>80</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C50" s="1">
         <v>743</v>
@@ -4560,7 +4560,7 @@
         <v>81</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C51" s="1">
         <v>743</v>
@@ -4635,7 +4635,7 @@
         <v>82</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C52" s="1">
         <v>743</v>
@@ -4710,7 +4710,7 @@
         <v>83</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C53" s="1">
         <v>743</v>
@@ -4785,7 +4785,7 @@
         <v>84</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C54" s="1">
         <v>743</v>
@@ -4860,7 +4860,7 @@
         <v>85</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C55" s="1">
         <v>743</v>
@@ -4935,7 +4935,7 @@
         <v>86</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C56" s="1">
         <v>743</v>
@@ -5010,7 +5010,7 @@
         <v>87</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C57" s="1">
         <v>743</v>
@@ -5085,7 +5085,7 @@
         <v>88</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C58" s="1">
         <v>743</v>
@@ -5160,7 +5160,7 @@
         <v>89</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C59" s="1">
         <v>743</v>
@@ -5235,7 +5235,7 @@
         <v>90</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C60" s="1">
         <v>743</v>
@@ -5310,7 +5310,7 @@
         <v>91</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C61" s="1">
         <v>743</v>
@@ -5385,7 +5385,7 @@
         <v>92</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C62" s="1">
         <v>869</v>
@@ -5454,7 +5454,7 @@
         <v>93</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C63" s="1">
         <v>869</v>
@@ -5523,7 +5523,7 @@
         <v>94</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C64" s="1">
         <v>869</v>
@@ -5595,7 +5595,7 @@
         <v>95</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C65" s="1">
         <v>869</v>
@@ -5664,7 +5664,7 @@
         <v>96</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C66" s="1">
         <v>869</v>
@@ -5733,7 +5733,7 @@
         <v>97</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C67" s="1">
         <v>869</v>
@@ -5802,7 +5802,7 @@
         <v>98</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C68" s="1">
         <v>409</v>
@@ -5877,7 +5877,7 @@
         <v>100</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C69" s="1">
         <v>409</v>
@@ -5952,7 +5952,7 @@
         <v>101</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C70" s="1">
         <v>409</v>
@@ -6027,7 +6027,7 @@
         <v>102</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C71" s="1">
         <v>409</v>
@@ -6102,7 +6102,7 @@
         <v>103</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C72" s="1">
         <v>409</v>
@@ -6177,7 +6177,7 @@
         <v>104</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C73" s="1">
         <v>409</v>
@@ -6252,7 +6252,7 @@
         <v>105</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C74" s="1">
         <v>409</v>
@@ -6327,7 +6327,7 @@
         <v>106</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C75" s="1">
         <v>409</v>
@@ -6402,7 +6402,7 @@
         <v>107</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C76" s="1">
         <v>409</v>
@@ -6477,7 +6477,7 @@
         <v>108</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C77" s="1">
         <v>409</v>
@@ -6552,7 +6552,7 @@
         <v>109</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C78" s="1">
         <v>409</v>
@@ -6627,7 +6627,7 @@
         <v>110</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C79" s="1">
         <v>409</v>
@@ -6699,7 +6699,7 @@
         <v>111</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C80" s="1">
         <v>409</v>
@@ -6771,7 +6771,7 @@
         <v>112</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C81" s="1">
         <v>409</v>
@@ -6843,7 +6843,7 @@
         <v>113</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C82" s="1">
         <v>409</v>
@@ -6915,7 +6915,7 @@
         <v>114</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C83" s="1">
         <v>409</v>
@@ -6987,7 +6987,7 @@
         <v>115</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C84" s="1">
         <v>409</v>
@@ -7059,7 +7059,7 @@
         <v>116</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C85" s="1">
         <v>409</v>
@@ -7131,7 +7131,7 @@
         <v>117</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C86" s="1">
         <v>409</v>
@@ -7203,7 +7203,7 @@
         <v>118</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C87" s="1">
         <v>409</v>
@@ -7275,7 +7275,7 @@
         <v>119</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C88" s="1">
         <v>409</v>
@@ -7347,7 +7347,7 @@
         <v>120</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C89" s="1">
         <v>409</v>
@@ -7419,7 +7419,7 @@
         <v>121</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C90" s="1">
         <v>409</v>
@@ -7491,7 +7491,7 @@
         <v>122</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C91" s="1">
         <v>409</v>
@@ -7563,7 +7563,7 @@
         <v>123</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C92" s="1">
         <v>409</v>
@@ -7632,7 +7632,7 @@
         <v>124</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C93" s="1">
         <v>409</v>
@@ -7704,7 +7704,7 @@
         <v>125</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C94" s="1">
         <v>409</v>
@@ -7773,7 +7773,7 @@
         <v>126</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C95" s="1">
         <v>409</v>
@@ -7845,7 +7845,7 @@
         <v>127</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C96" s="1">
         <v>409</v>
@@ -7917,7 +7917,7 @@
         <v>128</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C97" s="1">
         <v>409</v>
@@ -7989,7 +7989,7 @@
         <v>129</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C98" s="1">
         <v>409</v>
@@ -8058,7 +8058,7 @@
         <v>130</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C99" s="1">
         <v>409</v>
@@ -8130,7 +8130,7 @@
         <v>131</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C100" s="1">
         <v>409</v>
@@ -8202,7 +8202,7 @@
         <v>132</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C101" s="1">
         <v>409</v>

</xml_diff>